<commit_message>
Calculated task engagement vs gaze feature averages
</commit_message>
<xml_diff>
--- a/Recordings/SavedData/gaze_counts/gaze_counts_stats.xlsx
+++ b/Recordings/SavedData/gaze_counts/gaze_counts_stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonzacar\Documents\Python_Projects\vilearn_ml\Recordings\SavedData\gaze_counts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{529D0017-BE97-4F0F-B277-640B54C7FAB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02314F68-F080-429C-AAD2-7252A1941DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-13068" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{AC5CA040-C652-4AFF-9FF4-1E2C177083E0}"/>
+    <workbookView xWindow="57480" yWindow="2025" windowWidth="29040" windowHeight="17520" firstSheet="3" activeTab="4" xr2:uid="{AC5CA040-C652-4AFF-9FF4-1E2C177083E0}"/>
   </bookViews>
   <sheets>
     <sheet name="dyads_gaze_counts_stats_floorle" sheetId="6" r:id="rId1"/>
@@ -27,11 +27,11 @@
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">dyads_gaze_counts_stats_floorle!$A$1:$D$9</definedName>
     <definedName name="ExternalData_1" localSheetId="3" hidden="1">triads_gaze_counts_stats!$A$1:$J$9</definedName>
     <definedName name="ExternalData_1" localSheetId="2" hidden="1">triads_gaze_counts_stats_floorl!$A$1:$J$9</definedName>
-    <definedName name="ExternalData_2" localSheetId="4" hidden="1">COMPARISONS_full!$A$13:$D$21</definedName>
+    <definedName name="ExternalData_2" localSheetId="4" hidden="1">COMPARISONS_full!$A$26:$D$34</definedName>
     <definedName name="ExternalData_2" localSheetId="5" hidden="1">COMPARISONS_simple!$A$11:$D$14</definedName>
     <definedName name="ExternalData_3" localSheetId="4" hidden="1">COMPARISONS_full!$F$2:$O$10</definedName>
     <definedName name="ExternalData_3" localSheetId="5" hidden="1">COMPARISONS_simple!$F$2:$O$5</definedName>
-    <definedName name="ExternalData_4" localSheetId="4" hidden="1">COMPARISONS_full!$F$13:$O$21</definedName>
+    <definedName name="ExternalData_4" localSheetId="4" hidden="1">COMPARISONS_full!$F$26:$O$34</definedName>
     <definedName name="ExternalData_4" localSheetId="5" hidden="1">COMPARISONS_simple!$F$11:$O$14</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="24">
   <si>
     <t>count</t>
   </si>
@@ -163,6 +163,12 @@
   <si>
     <t>Triads All Gaze Configurations Counts</t>
   </si>
+  <si>
+    <t>Task Engagement</t>
+  </si>
+  <si>
+    <t>8 (P1) and  7(P2)</t>
+  </si>
 </sst>
 </file>
 
@@ -217,8 +223,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -228,10 +236,7 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -240,10 +245,13 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -503,10 +511,10 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B7A79111-A487-4750-80C5-6A5E0868B1AB}" name="dyads_gaze_counts_stats1115" displayName="dyads_gaze_counts_stats1115" ref="A11:D14" tableType="queryTable" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B7A79111-A487-4750-80C5-6A5E0868B1AB}" name="dyads_gaze_counts_stats1115" displayName="dyads_gaze_counts_stats1115" ref="A11:D14" tableType="queryTable" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A11:D14" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2DB397D4-FBEF-4722-8E17-B0AE91A266A7}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{2DB397D4-FBEF-4722-8E17-B0AE91A266A7}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{1B1CFC05-A671-4145-B60C-ADADD5D25B2E}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{240B3CA9-6AE8-48C0-872A-E819EA44F87C}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{9FC139DF-53B1-4D7E-AA17-6F6E692CA328}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
@@ -516,10 +524,10 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{7FDE0259-F321-4AAE-BB08-0BC2E5A737F7}" name="triads_gaze_counts_stats_floorlevel__21216" displayName="triads_gaze_counts_stats_floorlevel__21216" ref="F2:O5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{7FDE0259-F321-4AAE-BB08-0BC2E5A737F7}" name="triads_gaze_counts_stats_floorlevel__21216" displayName="triads_gaze_counts_stats_floorlevel__21216" ref="F2:O5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="F2:O5" xr:uid="{240E3FA1-9A53-416B-84DD-756B154FEAB1}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{F4E1600F-545A-4249-B39A-437021776FD3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{F4E1600F-545A-4249-B39A-437021776FD3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{F7E4BB1A-1081-423B-B73B-991F08FD0697}" uniqueName="2" name="Percentage_0_D1" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{22364F8F-4EDD-4D31-A8D7-15963C0A85C2}" uniqueName="3" name="Percentage_1_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{522654CA-D0D9-40EC-B2EA-7804300F44A8}" uniqueName="4" name="Percentage_2_D1_same" queryTableFieldId="4"/>
@@ -535,7 +543,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{9D6B5AA9-E372-4765-B2BD-764D74D5FB9B}" name="triads_gaze_counts_stats1317" displayName="triads_gaze_counts_stats1317" ref="F11:O14" tableType="queryTable" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{9D6B5AA9-E372-4765-B2BD-764D74D5FB9B}" name="triads_gaze_counts_stats1317" displayName="triads_gaze_counts_stats1317" ref="F11:O14" tableType="queryTable" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="F11:O14" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{881A3E44-7CB3-4944-8559-CA4EE2EA2E13}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="0"/>
@@ -618,8 +626,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}" name="dyads_gaze_counts_stats11" displayName="dyads_gaze_counts_stats11" ref="A13:D21" tableType="queryTable" totalsRowShown="0" headerRowDxfId="13">
-  <autoFilter ref="A13:D21" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}" name="dyads_gaze_counts_stats11" displayName="dyads_gaze_counts_stats11" ref="A26:D34" tableType="queryTable" totalsRowShown="0" headerRowDxfId="13">
+  <autoFilter ref="A26:D34" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{697A5396-42F9-401E-A8FF-32794083AD51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{1E92647F-C79B-46E0-A9E8-E79474C1F8D7}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
@@ -650,8 +658,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}" name="triads_gaze_counts_stats13" displayName="triads_gaze_counts_stats13" ref="F13:O21" tableType="queryTable" totalsRowShown="0" headerRowDxfId="9">
-  <autoFilter ref="F13:O21" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}" name="triads_gaze_counts_stats13" displayName="triads_gaze_counts_stats13" ref="F26:O34" tableType="queryTable" totalsRowShown="0" headerRowDxfId="9">
+  <autoFilter ref="F26:O34" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{A7232138-1AD4-4B88-874C-14C2C1081AAF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{0DA2B8B9-D9BD-4701-9A31-6287F8DD3C87}" uniqueName="2" name="Percentage_0_D1" queryTableFieldId="2"/>
@@ -672,7 +680,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{2D8EF511-1FB5-478B-A6CA-0226811E1394}" name="dyads_gaze_counts_stats_floorlevel__21014" displayName="dyads_gaze_counts_stats_floorlevel__21014" ref="A2:D5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="7">
   <autoFilter ref="A2:D5" xr:uid="{53B72080-B5EF-4656-81C3-34F5EEA880E8}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{BE4F5318-5C8B-45DA-8032-5DADA7840162}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{BE4F5318-5C8B-45DA-8032-5DADA7840162}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{2652FEA9-5E73-4A5C-B6C8-113038188438}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{7958EAAE-9C2F-413B-9BD5-DB1D396EB51B}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{3B2C7F5F-2941-4CD0-8CA3-F1750712FF7F}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
@@ -1910,7 +1918,1140 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7E8B623-2092-483D-AE1D-203C7F8C0744}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O34"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.6328125" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="F1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+    </row>
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>8</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>12</v>
+      </c>
+      <c r="H3">
+        <v>12</v>
+      </c>
+      <c r="I3">
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
+        <v>12</v>
+      </c>
+      <c r="M3">
+        <v>12</v>
+      </c>
+      <c r="N3">
+        <v>36</v>
+      </c>
+      <c r="O3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.26231101549635127</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.41657942882564714</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.32110955567800142</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0.50104232422697093</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.34624040590083749</v>
+      </c>
+      <c r="I4" s="2">
+        <v>4.92982431295916E-2</v>
+      </c>
+      <c r="J4" s="2">
+        <v>4.5391747969872054E-2</v>
+      </c>
+      <c r="K4" s="2">
+        <v>3.0321223225744172E-3</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1.0994218039000249E-2</v>
+      </c>
+      <c r="M4" s="2">
+        <v>4.4000938411153039E-2</v>
+      </c>
+      <c r="N4" s="2">
+        <v>1.8331718816717749E-2</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0.18523699103549615</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>0.24992946973577304</v>
+      </c>
+      <c r="C5">
+        <v>0.35784751123829683</v>
+      </c>
+      <c r="D5">
+        <v>0.16392518614238752</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5">
+        <v>0.26054281222722431</v>
+      </c>
+      <c r="H5">
+        <v>0.13235445182420261</v>
+      </c>
+      <c r="I5">
+        <v>0.10255200707982896</v>
+      </c>
+      <c r="J5">
+        <v>3.9226970720822534E-2</v>
+      </c>
+      <c r="K5">
+        <v>5.2243346309184188E-3</v>
+      </c>
+      <c r="L5">
+        <v>1.3443105388219948E-2</v>
+      </c>
+      <c r="M5">
+        <v>5.1742240123663248E-2</v>
+      </c>
+      <c r="N5">
+        <v>3.7740539951854349E-2</v>
+      </c>
+      <c r="O5">
+        <v>0.16384725382378432</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>6.1269397391523497E-2</v>
+      </c>
+      <c r="D6">
+        <v>2.0312897187622702E-2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6">
+        <v>7.2352499374113297E-2</v>
+      </c>
+      <c r="H6">
+        <v>6.1753568307602598E-2</v>
+      </c>
+      <c r="I6">
+        <v>2.3303233323619999E-4</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>1.2525487911446999E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>3.5382038027342376E-2</v>
+      </c>
+      <c r="C7">
+        <v>0.11655053300805086</v>
+      </c>
+      <c r="D7">
+        <v>0.26021459853210838</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7">
+        <v>0.3106709118389715</v>
+      </c>
+      <c r="H7">
+        <v>0.28949946569253909</v>
+      </c>
+      <c r="I7">
+        <v>5.85493699578905E-3</v>
+      </c>
+      <c r="J7">
+        <v>9.124732642850051E-3</v>
+      </c>
+      <c r="K7">
+        <v>5.9783186310978845E-5</v>
+      </c>
+      <c r="L7">
+        <v>2.3960813831572567E-4</v>
+      </c>
+      <c r="M7">
+        <v>9.4882269758518253E-3</v>
+      </c>
+      <c r="N7">
+        <v>9.6843835647532502E-4</v>
+      </c>
+      <c r="O7">
+        <v>7.3127231010150978E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>0.22857948021614283</v>
+      </c>
+      <c r="C8">
+        <v>0.30092235684370572</v>
+      </c>
+      <c r="D8">
+        <v>0.33465589316307282</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8">
+        <v>0.51288353428082045</v>
+      </c>
+      <c r="H8">
+        <v>0.39605324261495412</v>
+      </c>
+      <c r="I8">
+        <v>1.5870963408559299E-2</v>
+      </c>
+      <c r="J8">
+        <v>3.9735281245666998E-2</v>
+      </c>
+      <c r="K8">
+        <v>8.1645822658079996E-4</v>
+      </c>
+      <c r="L8">
+        <v>5.0768441624970502E-3</v>
+      </c>
+      <c r="M8">
+        <v>2.3150586858744701E-2</v>
+      </c>
+      <c r="N8">
+        <v>3.6143564423939999E-3</v>
+      </c>
+      <c r="O8">
+        <v>0.13609756918662891</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9">
+        <v>0.44209944596506179</v>
+      </c>
+      <c r="C9">
+        <v>0.70453046347983461</v>
+      </c>
+      <c r="D9">
+        <v>0.42453909723411004</v>
+      </c>
+      <c r="F9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9">
+        <v>0.65856523668963318</v>
+      </c>
+      <c r="H9">
+        <v>0.44998484531733857</v>
+      </c>
+      <c r="I9">
+        <v>3.44516995032507E-2</v>
+      </c>
+      <c r="J9">
+        <v>6.5372010805417546E-2</v>
+      </c>
+      <c r="K9">
+        <v>2.0985885766440751E-3</v>
+      </c>
+      <c r="L9">
+        <v>1.5985226546175176E-2</v>
+      </c>
+      <c r="M9">
+        <v>5.3753786521837627E-2</v>
+      </c>
+      <c r="N9">
+        <v>1.5557706900609876E-2</v>
+      </c>
+      <c r="O9">
+        <v>0.27345751604638319</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10">
+        <v>0.61670525133518239</v>
+      </c>
+      <c r="C10">
+        <v>0.97917870265523521</v>
+      </c>
+      <c r="D10">
+        <v>0.53251237946312224</v>
+      </c>
+      <c r="F10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10">
+        <v>0.93801339935916117</v>
+      </c>
+      <c r="H10">
+        <v>0.4730833898705053</v>
+      </c>
+      <c r="I10">
+        <v>0.36727029959108731</v>
+      </c>
+      <c r="J10">
+        <v>0.12702624469316859</v>
+      </c>
+      <c r="K10">
+        <v>1.6644152836742501E-2</v>
+      </c>
+      <c r="L10">
+        <v>3.7990257203185503E-2</v>
+      </c>
+      <c r="M10">
+        <v>0.1736079467784562</v>
+      </c>
+      <c r="N10">
+        <v>0.20167684316048479</v>
+      </c>
+      <c r="O10">
+        <v>0.71075690561628979</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>7</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>12</v>
+      </c>
+      <c r="H13">
+        <v>12</v>
+      </c>
+      <c r="I13">
+        <v>12</v>
+      </c>
+      <c r="J13">
+        <v>11</v>
+      </c>
+      <c r="K13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14">
+        <v>0.521034</v>
+      </c>
+      <c r="C14">
+        <v>0.46625</v>
+      </c>
+      <c r="D14">
+        <v>0.50947900000000002</v>
+      </c>
+      <c r="F14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14">
+        <v>0.41084100000000001</v>
+      </c>
+      <c r="H14">
+        <v>0.39891599999999999</v>
+      </c>
+      <c r="I14">
+        <v>0.38483899999999999</v>
+      </c>
+      <c r="J14">
+        <v>0.418989</v>
+      </c>
+      <c r="K14">
+        <v>0.42510700000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15">
+        <v>0.15657799999999999</v>
+      </c>
+      <c r="C15">
+        <v>0.158251</v>
+      </c>
+      <c r="D15">
+        <v>4.9550999999999998E-2</v>
+      </c>
+      <c r="F15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15">
+        <v>0.151505</v>
+      </c>
+      <c r="H15">
+        <v>0.132773</v>
+      </c>
+      <c r="I15">
+        <v>0.15337999999999999</v>
+      </c>
+      <c r="J15">
+        <v>0.155973</v>
+      </c>
+      <c r="K15">
+        <v>0.21804999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16">
+        <v>0.308894</v>
+      </c>
+      <c r="C16">
+        <v>0.21893099999999999</v>
+      </c>
+      <c r="D16">
+        <v>0.474441</v>
+      </c>
+      <c r="F16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16">
+        <v>8.0060000000000006E-2</v>
+      </c>
+      <c r="H16">
+        <v>0.113082</v>
+      </c>
+      <c r="I16">
+        <v>3.5699000000000002E-2</v>
+      </c>
+      <c r="J16">
+        <v>0.129576</v>
+      </c>
+      <c r="K16">
+        <v>1.5138E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A17" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="B17">
+        <v>0.43718699999999999</v>
+      </c>
+      <c r="C17">
+        <v>0.35931800000000003</v>
+      </c>
+      <c r="D17">
+        <v>0.49196000000000001</v>
+      </c>
+      <c r="F17" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="G17">
+        <v>0.311083</v>
+      </c>
+      <c r="H17">
+        <v>0.32530500000000001</v>
+      </c>
+      <c r="I17">
+        <v>0.35852899999999999</v>
+      </c>
+      <c r="J17">
+        <v>0.34237499999999998</v>
+      </c>
+      <c r="K17">
+        <v>0.35978100000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A18" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="B18">
+        <v>0.51513399999999998</v>
+      </c>
+      <c r="C18">
+        <v>0.52607899999999996</v>
+      </c>
+      <c r="D18">
+        <v>0.50947900000000002</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="G18">
+        <v>0.44086500000000001</v>
+      </c>
+      <c r="H18">
+        <v>0.41766300000000001</v>
+      </c>
+      <c r="I18">
+        <v>0.42343199999999998</v>
+      </c>
+      <c r="J18">
+        <v>0.44447399999999998</v>
+      </c>
+      <c r="K18">
+        <v>0.43415100000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A19" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="B19">
+        <v>0.57845899999999995</v>
+      </c>
+      <c r="C19">
+        <v>0.58607500000000001</v>
+      </c>
+      <c r="D19">
+        <v>0.52699799999999997</v>
+      </c>
+      <c r="F19" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="G19">
+        <v>0.49920100000000001</v>
+      </c>
+      <c r="H19">
+        <v>0.46976899999999999</v>
+      </c>
+      <c r="I19">
+        <v>0.46191700000000002</v>
+      </c>
+      <c r="J19">
+        <v>0.516652</v>
+      </c>
+      <c r="K19">
+        <v>0.55061400000000005</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20">
+        <v>0.79192099999999999</v>
+      </c>
+      <c r="C20">
+        <v>0.62071100000000001</v>
+      </c>
+      <c r="D20">
+        <v>0.54451700000000003</v>
+      </c>
+      <c r="F20" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20">
+        <v>0.62566200000000005</v>
+      </c>
+      <c r="H20">
+        <v>0.58872800000000003</v>
+      </c>
+      <c r="I20">
+        <v>0.61673500000000003</v>
+      </c>
+      <c r="J20">
+        <v>0.67054999999999998</v>
+      </c>
+      <c r="K20">
+        <v>0.72725600000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A25" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="F25" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+    </row>
+    <row r="26" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="N26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B27">
+        <v>11</v>
+      </c>
+      <c r="C27">
+        <v>11</v>
+      </c>
+      <c r="D27">
+        <v>11</v>
+      </c>
+      <c r="F27" t="s">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>14</v>
+      </c>
+      <c r="H27">
+        <v>14</v>
+      </c>
+      <c r="I27">
+        <v>14</v>
+      </c>
+      <c r="J27">
+        <v>14</v>
+      </c>
+      <c r="K27">
+        <v>14</v>
+      </c>
+      <c r="L27">
+        <v>14</v>
+      </c>
+      <c r="M27">
+        <v>14</v>
+      </c>
+      <c r="N27">
+        <v>42</v>
+      </c>
+      <c r="O27">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" s="2">
+        <v>0.19340415942472544</v>
+      </c>
+      <c r="C28" s="2">
+        <v>0.51837748819620566</v>
+      </c>
+      <c r="D28" s="2">
+        <v>0.28821835237906868</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G28" s="2">
+        <v>0.5440218639511919</v>
+      </c>
+      <c r="H28" s="2">
+        <v>0.3227610920575627</v>
+      </c>
+      <c r="I28" s="2">
+        <v>4.2979385297251829E-2</v>
+      </c>
+      <c r="J28" s="2">
+        <v>3.9383873367815014E-2</v>
+      </c>
+      <c r="K28" s="2">
+        <v>2.5989619907780719E-3</v>
+      </c>
+      <c r="L28" s="2">
+        <v>9.4665509621451212E-3</v>
+      </c>
+      <c r="M28" s="2">
+        <v>3.8788272373255224E-2</v>
+      </c>
+      <c r="N28" s="2">
+        <v>1.6084941111800099E-2</v>
+      </c>
+      <c r="O28" s="2">
+        <v>0.16825034877405864</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29">
+        <v>0.24021453920877969</v>
+      </c>
+      <c r="C29">
+        <v>0.35065687915662397</v>
+      </c>
+      <c r="D29">
+        <v>0.15653864357905634</v>
+      </c>
+      <c r="F29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29">
+        <v>0.26491513587477228</v>
+      </c>
+      <c r="H29">
+        <v>0.13777553120139505</v>
+      </c>
+      <c r="I29">
+        <v>9.5709469195713076E-2</v>
+      </c>
+      <c r="J29">
+        <v>3.91826918136109E-2</v>
+      </c>
+      <c r="K29">
+        <v>4.9302140461371892E-3</v>
+      </c>
+      <c r="L29">
+        <v>1.2961792874198175E-2</v>
+      </c>
+      <c r="M29">
+        <v>4.943842925318119E-2</v>
+      </c>
+      <c r="N29">
+        <v>3.5329150299028167E-2</v>
+      </c>
+      <c r="O29">
+        <v>0.1580123822126264</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30">
+        <v>0</v>
+      </c>
+      <c r="C30">
+        <v>6.1269397391523497E-2</v>
+      </c>
+      <c r="D30">
+        <v>2.0312897187622702E-2</v>
+      </c>
+      <c r="F30" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30">
+        <v>7.2352499374113297E-2</v>
+      </c>
+      <c r="H30">
+        <v>6.1753568307602598E-2</v>
+      </c>
+      <c r="I30">
+        <v>2.3303233323619999E-4</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30">
+        <v>0</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>1.2525487911446999E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31">
+        <v>6.5674775810715003E-4</v>
+      </c>
+      <c r="C31">
+        <v>0.21276105112635874</v>
+      </c>
+      <c r="D31">
+        <v>0.22075770732100614</v>
+      </c>
+      <c r="F31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31">
+        <v>0.33369444307812707</v>
+      </c>
+      <c r="H31">
+        <v>0.25459334719845034</v>
+      </c>
+      <c r="I31">
+        <v>3.6419178573711504E-3</v>
+      </c>
+      <c r="J31">
+        <v>4.4573895537424755E-3</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+      <c r="L31">
+        <v>1.3597193490997694E-4</v>
+      </c>
+      <c r="M31">
+        <v>8.9974080943096748E-3</v>
+      </c>
+      <c r="N31">
+        <v>7.2856560004650001E-5</v>
+      </c>
+      <c r="O31">
+        <v>6.2172568250083125E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>15</v>
+      </c>
+      <c r="B32">
+        <v>4.7006583984075902E-2</v>
+      </c>
+      <c r="C32">
+        <v>0.66533966212422802</v>
+      </c>
+      <c r="D32">
+        <v>0.28765375389169601</v>
+      </c>
+      <c r="F32" t="s">
+        <v>15</v>
+      </c>
+      <c r="G32">
+        <v>0.57159295554916678</v>
+      </c>
+      <c r="H32">
+        <v>0.35354368307406436</v>
+      </c>
+      <c r="I32">
+        <v>1.2490366451266201E-2</v>
+      </c>
+      <c r="J32">
+        <v>3.68289537607559E-2</v>
+      </c>
+      <c r="K32">
+        <v>6.3038046787094993E-4</v>
+      </c>
+      <c r="L32">
+        <v>1.8612768646099E-3</v>
+      </c>
+      <c r="M32">
+        <v>1.6624045871298551E-2</v>
+      </c>
+      <c r="N32">
+        <v>3.2330596008071501E-3</v>
+      </c>
+      <c r="O32">
+        <v>0.12491664830181609</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33">
+        <v>0.33959342381557356</v>
+      </c>
+      <c r="C33">
+        <v>0.77910022416137725</v>
+      </c>
+      <c r="D33">
+        <v>0.37788519073501603</v>
+      </c>
+      <c r="F33" t="s">
+        <v>16</v>
+      </c>
+      <c r="G33">
+        <v>0.71964111242898787</v>
+      </c>
+      <c r="H33">
+        <v>0.44348306085627381</v>
+      </c>
+      <c r="I33">
+        <v>3.1945389594186149E-2</v>
+      </c>
+      <c r="J33">
+        <v>5.9883995345627897E-2</v>
+      </c>
+      <c r="K33">
+        <v>1.2911585032818499E-3</v>
+      </c>
+      <c r="L33">
+        <v>1.31876466736869E-2</v>
+      </c>
+      <c r="M33">
+        <v>4.2081899741738225E-2</v>
+      </c>
+      <c r="N33">
+        <v>9.2926703488600253E-3</v>
+      </c>
+      <c r="O33">
+        <v>0.23941064492750608</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>17</v>
+      </c>
+      <c r="B34">
+        <v>0.61670525133518239</v>
+      </c>
+      <c r="C34">
+        <v>0.97917870265523521</v>
+      </c>
+      <c r="D34">
+        <v>0.53251237946312224</v>
+      </c>
+      <c r="F34" t="s">
+        <v>17</v>
+      </c>
+      <c r="G34">
+        <v>0.93801339935916117</v>
+      </c>
+      <c r="H34">
+        <v>0.4730833898705053</v>
+      </c>
+      <c r="I34">
+        <v>0.36727029959108731</v>
+      </c>
+      <c r="J34">
+        <v>0.12702624469316859</v>
+      </c>
+      <c r="K34">
+        <v>1.6644152836742501E-2</v>
+      </c>
+      <c r="L34">
+        <v>3.7990257203185503E-2</v>
+      </c>
+      <c r="M34">
+        <v>0.1736079467784562</v>
+      </c>
+      <c r="N34">
+        <v>0.20167684316048479</v>
+      </c>
+      <c r="O34">
+        <v>0.71075690561628979</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="F1:O1"/>
+    <mergeCell ref="F25:O25"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="4">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95E10051-0AE9-4412-9EB8-15AF454AC83C}">
+  <dimension ref="A1:O14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
@@ -2046,7 +3187,7 @@
         <v>0.41657942882564714</v>
       </c>
       <c r="D4" s="2">
-        <v>0.32110955567800142</v>
+        <v>0.32110955567800098</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>11</v>
@@ -2090,7 +3231,7 @@
         <v>0.35784751123829683</v>
       </c>
       <c r="D5">
-        <v>0.16392518614238752</v>
+        <v>0.16392518614238799</v>
       </c>
       <c r="F5" t="s">
         <v>12</v>
@@ -2122,887 +3263,6 @@
       <c r="O5">
         <v>0.16384725382378432</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>6.1269397391523497E-2</v>
-      </c>
-      <c r="D6">
-        <v>2.0312897187622702E-2</v>
-      </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6">
-        <v>7.2352499374113297E-2</v>
-      </c>
-      <c r="H6">
-        <v>6.1753568307602598E-2</v>
-      </c>
-      <c r="I6">
-        <v>2.3303233323619999E-4</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>1.2525487911446999E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7">
-        <v>3.5382038027342376E-2</v>
-      </c>
-      <c r="C7">
-        <v>0.11655053300805086</v>
-      </c>
-      <c r="D7">
-        <v>0.26021459853210838</v>
-      </c>
-      <c r="F7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7">
-        <v>0.3106709118389715</v>
-      </c>
-      <c r="H7">
-        <v>0.28949946569253909</v>
-      </c>
-      <c r="I7">
-        <v>5.85493699578905E-3</v>
-      </c>
-      <c r="J7">
-        <v>9.124732642850051E-3</v>
-      </c>
-      <c r="K7">
-        <v>5.9783186310978845E-5</v>
-      </c>
-      <c r="L7">
-        <v>2.3960813831572567E-4</v>
-      </c>
-      <c r="M7">
-        <v>9.4882269758518253E-3</v>
-      </c>
-      <c r="N7">
-        <v>9.6843835647532502E-4</v>
-      </c>
-      <c r="O7">
-        <v>7.3127231010150978E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8">
-        <v>0.22857948021614283</v>
-      </c>
-      <c r="C8">
-        <v>0.30092235684370572</v>
-      </c>
-      <c r="D8">
-        <v>0.33465589316307282</v>
-      </c>
-      <c r="F8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8">
-        <v>0.51288353428082045</v>
-      </c>
-      <c r="H8">
-        <v>0.39605324261495412</v>
-      </c>
-      <c r="I8">
-        <v>1.5870963408559299E-2</v>
-      </c>
-      <c r="J8">
-        <v>3.9735281245666998E-2</v>
-      </c>
-      <c r="K8">
-        <v>8.1645822658079996E-4</v>
-      </c>
-      <c r="L8">
-        <v>5.0768441624970502E-3</v>
-      </c>
-      <c r="M8">
-        <v>2.3150586858744701E-2</v>
-      </c>
-      <c r="N8">
-        <v>3.6143564423939999E-3</v>
-      </c>
-      <c r="O8">
-        <v>0.13609756918662891</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9">
-        <v>0.44209944596506179</v>
-      </c>
-      <c r="C9">
-        <v>0.70453046347983461</v>
-      </c>
-      <c r="D9">
-        <v>0.42453909723411004</v>
-      </c>
-      <c r="F9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9">
-        <v>0.65856523668963318</v>
-      </c>
-      <c r="H9">
-        <v>0.44998484531733857</v>
-      </c>
-      <c r="I9">
-        <v>3.44516995032507E-2</v>
-      </c>
-      <c r="J9">
-        <v>6.5372010805417546E-2</v>
-      </c>
-      <c r="K9">
-        <v>2.0985885766440751E-3</v>
-      </c>
-      <c r="L9">
-        <v>1.5985226546175176E-2</v>
-      </c>
-      <c r="M9">
-        <v>5.3753786521837627E-2</v>
-      </c>
-      <c r="N9">
-        <v>1.5557706900609876E-2</v>
-      </c>
-      <c r="O9">
-        <v>0.27345751604638319</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10">
-        <v>0.61670525133518239</v>
-      </c>
-      <c r="C10">
-        <v>0.97917870265523521</v>
-      </c>
-      <c r="D10">
-        <v>0.53251237946312224</v>
-      </c>
-      <c r="F10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10">
-        <v>0.93801339935916117</v>
-      </c>
-      <c r="H10">
-        <v>0.4730833898705053</v>
-      </c>
-      <c r="I10">
-        <v>0.36727029959108731</v>
-      </c>
-      <c r="J10">
-        <v>0.12702624469316859</v>
-      </c>
-      <c r="K10">
-        <v>1.6644152836742501E-2</v>
-      </c>
-      <c r="L10">
-        <v>3.7990257203185503E-2</v>
-      </c>
-      <c r="M10">
-        <v>0.1736079467784562</v>
-      </c>
-      <c r="N10">
-        <v>0.20167684316048479</v>
-      </c>
-      <c r="O10">
-        <v>0.71075690561628979</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="F12" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-    </row>
-    <row r="13" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="N13" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B14">
-        <v>11</v>
-      </c>
-      <c r="C14">
-        <v>11</v>
-      </c>
-      <c r="D14">
-        <v>11</v>
-      </c>
-      <c r="F14" t="s">
-        <v>0</v>
-      </c>
-      <c r="G14">
-        <v>14</v>
-      </c>
-      <c r="H14">
-        <v>14</v>
-      </c>
-      <c r="I14">
-        <v>14</v>
-      </c>
-      <c r="J14">
-        <v>14</v>
-      </c>
-      <c r="K14">
-        <v>14</v>
-      </c>
-      <c r="L14">
-        <v>14</v>
-      </c>
-      <c r="M14">
-        <v>14</v>
-      </c>
-      <c r="N14">
-        <v>42</v>
-      </c>
-      <c r="O14">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="2">
-        <v>0.19340415942472544</v>
-      </c>
-      <c r="C15" s="2">
-        <v>0.51837748819620566</v>
-      </c>
-      <c r="D15" s="2">
-        <v>0.28821835237906868</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" s="2">
-        <v>0.5440218639511919</v>
-      </c>
-      <c r="H15" s="2">
-        <v>0.3227610920575627</v>
-      </c>
-      <c r="I15" s="2">
-        <v>4.2979385297251829E-2</v>
-      </c>
-      <c r="J15" s="2">
-        <v>3.9383873367815014E-2</v>
-      </c>
-      <c r="K15" s="2">
-        <v>2.5989619907780719E-3</v>
-      </c>
-      <c r="L15" s="2">
-        <v>9.4665509621451212E-3</v>
-      </c>
-      <c r="M15" s="2">
-        <v>3.8788272373255224E-2</v>
-      </c>
-      <c r="N15" s="2">
-        <v>1.6084941111800099E-2</v>
-      </c>
-      <c r="O15" s="2">
-        <v>0.16825034877405864</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16">
-        <v>0.24021453920877969</v>
-      </c>
-      <c r="C16">
-        <v>0.35065687915662397</v>
-      </c>
-      <c r="D16">
-        <v>0.15653864357905634</v>
-      </c>
-      <c r="F16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16">
-        <v>0.26491513587477228</v>
-      </c>
-      <c r="H16">
-        <v>0.13777553120139505</v>
-      </c>
-      <c r="I16">
-        <v>9.5709469195713076E-2</v>
-      </c>
-      <c r="J16">
-        <v>3.91826918136109E-2</v>
-      </c>
-      <c r="K16">
-        <v>4.9302140461371892E-3</v>
-      </c>
-      <c r="L16">
-        <v>1.2961792874198175E-2</v>
-      </c>
-      <c r="M16">
-        <v>4.943842925318119E-2</v>
-      </c>
-      <c r="N16">
-        <v>3.5329150299028167E-2</v>
-      </c>
-      <c r="O16">
-        <v>0.1580123822126264</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17">
-        <v>0</v>
-      </c>
-      <c r="C17">
-        <v>6.1269397391523497E-2</v>
-      </c>
-      <c r="D17">
-        <v>2.0312897187622702E-2</v>
-      </c>
-      <c r="F17" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17">
-        <v>7.2352499374113297E-2</v>
-      </c>
-      <c r="H17">
-        <v>6.1753568307602598E-2</v>
-      </c>
-      <c r="I17">
-        <v>2.3303233323619999E-4</v>
-      </c>
-      <c r="J17">
-        <v>0</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <v>0</v>
-      </c>
-      <c r="O17">
-        <v>1.2525487911446999E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18">
-        <v>6.5674775810715003E-4</v>
-      </c>
-      <c r="C18">
-        <v>0.21276105112635874</v>
-      </c>
-      <c r="D18">
-        <v>0.22075770732100614</v>
-      </c>
-      <c r="F18" t="s">
-        <v>14</v>
-      </c>
-      <c r="G18">
-        <v>0.33369444307812707</v>
-      </c>
-      <c r="H18">
-        <v>0.25459334719845034</v>
-      </c>
-      <c r="I18">
-        <v>3.6419178573711504E-3</v>
-      </c>
-      <c r="J18">
-        <v>4.4573895537424755E-3</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>1.3597193490997694E-4</v>
-      </c>
-      <c r="M18">
-        <v>8.9974080943096748E-3</v>
-      </c>
-      <c r="N18">
-        <v>7.2856560004650001E-5</v>
-      </c>
-      <c r="O18">
-        <v>6.2172568250083125E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19">
-        <v>4.7006583984075902E-2</v>
-      </c>
-      <c r="C19">
-        <v>0.66533966212422802</v>
-      </c>
-      <c r="D19">
-        <v>0.28765375389169601</v>
-      </c>
-      <c r="F19" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19">
-        <v>0.57159295554916678</v>
-      </c>
-      <c r="H19">
-        <v>0.35354368307406436</v>
-      </c>
-      <c r="I19">
-        <v>1.2490366451266201E-2</v>
-      </c>
-      <c r="J19">
-        <v>3.68289537607559E-2</v>
-      </c>
-      <c r="K19">
-        <v>6.3038046787094993E-4</v>
-      </c>
-      <c r="L19">
-        <v>1.8612768646099E-3</v>
-      </c>
-      <c r="M19">
-        <v>1.6624045871298551E-2</v>
-      </c>
-      <c r="N19">
-        <v>3.2330596008071501E-3</v>
-      </c>
-      <c r="O19">
-        <v>0.12491664830181609</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20">
-        <v>0.33959342381557356</v>
-      </c>
-      <c r="C20">
-        <v>0.77910022416137725</v>
-      </c>
-      <c r="D20">
-        <v>0.37788519073501603</v>
-      </c>
-      <c r="F20" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20">
-        <v>0.71964111242898787</v>
-      </c>
-      <c r="H20">
-        <v>0.44348306085627381</v>
-      </c>
-      <c r="I20">
-        <v>3.1945389594186149E-2</v>
-      </c>
-      <c r="J20">
-        <v>5.9883995345627897E-2</v>
-      </c>
-      <c r="K20">
-        <v>1.2911585032818499E-3</v>
-      </c>
-      <c r="L20">
-        <v>1.31876466736869E-2</v>
-      </c>
-      <c r="M20">
-        <v>4.2081899741738225E-2</v>
-      </c>
-      <c r="N20">
-        <v>9.2926703488600253E-3</v>
-      </c>
-      <c r="O20">
-        <v>0.23941064492750608</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21">
-        <v>0.61670525133518239</v>
-      </c>
-      <c r="C21">
-        <v>0.97917870265523521</v>
-      </c>
-      <c r="D21">
-        <v>0.53251237946312224</v>
-      </c>
-      <c r="F21" t="s">
-        <v>17</v>
-      </c>
-      <c r="G21">
-        <v>0.93801339935916117</v>
-      </c>
-      <c r="H21">
-        <v>0.4730833898705053</v>
-      </c>
-      <c r="I21">
-        <v>0.36727029959108731</v>
-      </c>
-      <c r="J21">
-        <v>0.12702624469316859</v>
-      </c>
-      <c r="K21">
-        <v>1.6644152836742501E-2</v>
-      </c>
-      <c r="L21">
-        <v>3.7990257203185503E-2</v>
-      </c>
-      <c r="M21">
-        <v>0.1736079467784562</v>
-      </c>
-      <c r="N21">
-        <v>0.20167684316048479</v>
-      </c>
-      <c r="O21">
-        <v>0.71075690561628979</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="F1:O1"/>
-    <mergeCell ref="F12:O12"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="4">
-    <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
-    <tablePart r:id="rId4"/>
-    <tablePart r:id="rId5"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95E10051-0AE9-4412-9EB8-15AF454AC83C}">
-  <dimension ref="A1:O25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="F1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-    </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3">
-        <v>8</v>
-      </c>
-      <c r="C3">
-        <v>8</v>
-      </c>
-      <c r="D3">
-        <v>8</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>12</v>
-      </c>
-      <c r="H3">
-        <v>12</v>
-      </c>
-      <c r="I3">
-        <v>12</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>12</v>
-      </c>
-      <c r="L3">
-        <v>12</v>
-      </c>
-      <c r="M3">
-        <v>12</v>
-      </c>
-      <c r="N3">
-        <v>36</v>
-      </c>
-      <c r="O3">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2">
-        <v>0.26231101549635127</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.41657942882564714</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0.32110955567800098</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0.50104232422697093</v>
-      </c>
-      <c r="H4" s="2">
-        <v>0.34624040590083749</v>
-      </c>
-      <c r="I4" s="2">
-        <v>4.92982431295916E-2</v>
-      </c>
-      <c r="J4" s="2">
-        <v>4.5391747969872054E-2</v>
-      </c>
-      <c r="K4" s="2">
-        <v>3.0321223225744172E-3</v>
-      </c>
-      <c r="L4" s="2">
-        <v>1.0994218039000249E-2</v>
-      </c>
-      <c r="M4" s="2">
-        <v>4.4000938411153039E-2</v>
-      </c>
-      <c r="N4" s="2">
-        <v>1.8331718816717749E-2</v>
-      </c>
-      <c r="O4" s="2">
-        <v>0.18523699103549615</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5">
-        <v>0.24992946973577304</v>
-      </c>
-      <c r="C5">
-        <v>0.35784751123829683</v>
-      </c>
-      <c r="D5">
-        <v>0.16392518614238799</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5">
-        <v>0.26054281222722431</v>
-      </c>
-      <c r="H5">
-        <v>0.13235445182420261</v>
-      </c>
-      <c r="I5">
-        <v>0.10255200707982896</v>
-      </c>
-      <c r="J5">
-        <v>3.9226970720822534E-2</v>
-      </c>
-      <c r="K5">
-        <v>5.2243346309184188E-3</v>
-      </c>
-      <c r="L5">
-        <v>1.3443105388219948E-2</v>
-      </c>
-      <c r="M5">
-        <v>5.1742240123663248E-2</v>
-      </c>
-      <c r="N5">
-        <v>3.7740539951854349E-2</v>
-      </c>
-      <c r="O5">
-        <v>0.16384725382378432</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A6" s="5"/>
-      <c r="F6" s="5"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A7" s="5"/>
-      <c r="F7" s="5"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A8" s="5"/>
-      <c r="F8" s="5"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
@@ -3069,7 +3329,7 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A12" s="5" t="s">
+      <c r="A12" t="s">
         <v>0</v>
       </c>
       <c r="B12">
@@ -3081,7 +3341,7 @@
       <c r="D12">
         <v>11</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" t="s">
         <v>0</v>
       </c>
       <c r="G12">
@@ -3113,7 +3373,7 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="2">
@@ -3125,7 +3385,7 @@
       <c r="D13" s="2">
         <v>0.28821835237906868</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G13" s="2">
@@ -3157,7 +3417,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
       <c r="B14">
@@ -3169,7 +3429,7 @@
       <c r="D14">
         <v>0.156538643579056</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" t="s">
         <v>12</v>
       </c>
       <c r="G14">
@@ -3199,50 +3459,6 @@
       <c r="O14">
         <v>0.1580123822126264</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A15" s="5"/>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A16" s="5"/>
-      <c r="F16" s="5"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="5"/>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="5"/>
-      <c r="F18" s="5"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="5"/>
-      <c r="F19" s="5"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="5"/>
-      <c r="F20" s="5"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="5"/>
-      <c r="F21" s="5"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="5"/>
-      <c r="F22" s="5"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="5"/>
-      <c r="F23" s="5"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="5"/>
-      <c r="F24" s="5"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="5"/>
-      <c r="F25" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
some modifications on the excel files
</commit_message>
<xml_diff>
--- a/Recordings/SavedData/gaze_counts/gaze_counts_stats.xlsx
+++ b/Recordings/SavedData/gaze_counts/gaze_counts_stats.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonzacar\Documents\Python_Projects\vilearn_ml\Recordings\SavedData\gaze_counts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\Recordings\SavedData\gaze_counts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9856F2-67D9-4E76-BCD3-1104A5ABD986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B8BF9D-9A6F-4D0B-A0D9-69B603D691C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="3" activeTab="4" xr2:uid="{AC5CA040-C652-4AFF-9FF4-1E2C177083E0}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="34">
   <si>
     <t>count</t>
   </si>
@@ -164,17 +164,47 @@
     <t>Triads All Gaze Configurations Counts</t>
   </si>
   <si>
-    <t>Task Engagement</t>
+    <t>8 (P1) and  7(P2)</t>
   </si>
   <si>
-    <t>8 (P1) and  7(P2)</t>
+    <t>Dyads Task Engagement</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>0_D1</t>
+  </si>
+  <si>
+    <t>1_D1</t>
+  </si>
+  <si>
+    <t>2_D1_same</t>
+  </si>
+  <si>
+    <t>2_D1_diff</t>
+  </si>
+  <si>
+    <t>3_D1</t>
+  </si>
+  <si>
+    <t>MG_D1</t>
+  </si>
+  <si>
+    <t>MG_D0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Triads Task Engagement </t>
+  </si>
+  <si>
+    <t>occourance in data(frm the above table)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -186,6 +216,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -211,27 +247,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="24">
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -501,7 +554,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F2B61F29-D93E-40BF-9C00-A67FEE87AFBC}" name="dyads_gaze_counts_stats_floorlevel__2" displayName="dyads_gaze_counts_stats_floorlevel__2" ref="A1:D9" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D9" xr:uid="{F2B61F29-D93E-40BF-9C00-A67FEE87AFBC}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{1EF82F3E-E46D-4D57-AE2E-FBC34C0DC041}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{1EF82F3E-E46D-4D57-AE2E-FBC34C0DC041}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="23"/>
     <tableColumn id="2" xr3:uid="{E0C558AE-F11F-4F96-96F9-0EB76F305EF5}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{ED6412B7-2EA6-4D46-89B2-8B626D591E60}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{150419C3-519B-492D-9B69-3FE260734E3B}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
@@ -511,10 +564,70 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B7A79111-A487-4750-80C5-6A5E0868B1AB}" name="dyads_gaze_counts_stats1115" displayName="dyads_gaze_counts_stats1115" ref="A11:D14" tableType="queryTable" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{23645723-A5D6-4262-B4C5-8C07E70BAE46}" name="Table2" displayName="Table2" ref="F12:M20" totalsRowShown="0">
+  <autoFilter ref="F12:M20" xr:uid="{23645723-A5D6-4262-B4C5-8C07E70BAE46}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{3433C2BC-B596-406B-831B-1FCD04621CFB}" name="Triads Task Engagement " dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{3B4B09E6-C745-4E93-BCE5-84021833960A}" name="0_D1"/>
+    <tableColumn id="3" xr3:uid="{D7BBC687-A0FE-40CF-A947-24B38B24B509}" name="1_D1"/>
+    <tableColumn id="4" xr3:uid="{83D61E69-C3DA-463C-AEF1-AB6CABFA1E1A}" name="2_D1_same"/>
+    <tableColumn id="5" xr3:uid="{B9955F04-7183-4478-99E4-47F1333A60A8}" name="2_D1_diff"/>
+    <tableColumn id="6" xr3:uid="{8AF578C5-2768-4224-8093-AA75F4088488}" name="3_D1"/>
+    <tableColumn id="7" xr3:uid="{EA5982D5-5735-478E-A8ED-0B3310CA9EDD}" name="MG_D1"/>
+    <tableColumn id="8" xr3:uid="{B9308BEB-7CF0-4726-9E23-8345BBD94D21}" name="MG_D0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A510564C-C2D5-4AD7-AD14-41BFBB76DE36}" name="Table24" displayName="Table24" ref="F43:M52" totalsRowShown="0">
+  <autoFilter ref="F43:M52" xr:uid="{A510564C-C2D5-4AD7-AD14-41BFBB76DE36}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{E183747D-84EC-4B87-8B67-E890AA975C40}" name="Triads Task Engagement " dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{7CA9C56E-375C-486B-99F9-80FF0325D85D}" name="0_D1"/>
+    <tableColumn id="3" xr3:uid="{5C20202F-D733-428A-AC29-E4F5067DB622}" name="1_D1"/>
+    <tableColumn id="4" xr3:uid="{8D0A5DC7-881B-471C-A585-FE7AF5148EAB}" name="2_D1_same"/>
+    <tableColumn id="5" xr3:uid="{7377F3F8-6BE0-48DB-8B63-B504ED9284B5}" name="2_D1_diff"/>
+    <tableColumn id="6" xr3:uid="{B81B54C4-3A21-46A2-93ED-41F8BB721F05}" name="3_D1"/>
+    <tableColumn id="7" xr3:uid="{EF9FA6C8-96C1-4541-A081-69DCFF7BF674}" name="MG_D1"/>
+    <tableColumn id="8" xr3:uid="{B949E979-B8BA-4A11-BF74-7921F8A8E113}" name="MG_D0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{52FDEAE4-DA20-42E7-BD4C-0CFED2DF38A9}" name="Table15" displayName="Table15" ref="A43:D52" totalsRowShown="0">
+  <autoFilter ref="A43:D52" xr:uid="{52FDEAE4-DA20-42E7-BD4C-0CFED2DF38A9}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{EF80BF77-87EE-4D56-9212-F2FD4E35E546}" name="Dyads Task Engagement" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{BA5FD875-4083-43AE-9B5B-2031AD0121FC}" name="MG"/>
+    <tableColumn id="3" xr3:uid="{7058BAA9-7A1F-4B3E-BB9F-49F68EA4D5DF}" name="0_D1"/>
+    <tableColumn id="4" xr3:uid="{B5873DF6-2681-46FC-B69E-F58AF37B98E9}" name="1_D1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{2D8EF511-1FB5-478B-A6CA-0226811E1394}" name="dyads_gaze_counts_stats_floorlevel__21014" displayName="dyads_gaze_counts_stats_floorlevel__21014" ref="A2:D5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="11">
+  <autoFilter ref="A2:D5" xr:uid="{53B72080-B5EF-4656-81C3-34F5EEA880E8}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{BE4F5318-5C8B-45DA-8032-5DADA7840162}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{2652FEA9-5E73-4A5C-B6C8-113038188438}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
+    <tableColumn id="3" xr3:uid="{7958EAAE-9C2F-413B-9BD5-DB1D396EB51B}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
+    <tableColumn id="4" xr3:uid="{3B2C7F5F-2941-4CD0-8CA3-F1750712FF7F}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B7A79111-A487-4750-80C5-6A5E0868B1AB}" name="dyads_gaze_counts_stats1115" displayName="dyads_gaze_counts_stats1115" ref="A11:D14" tableType="queryTable" totalsRowShown="0" headerRowDxfId="9">
   <autoFilter ref="A11:D14" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2DB397D4-FBEF-4722-8E17-B0AE91A266A7}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{2DB397D4-FBEF-4722-8E17-B0AE91A266A7}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{1B1CFC05-A671-4145-B60C-ADADD5D25B2E}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{240B3CA9-6AE8-48C0-872A-E819EA44F87C}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{9FC139DF-53B1-4D7E-AA17-6F6E692CA328}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
@@ -523,11 +636,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{7FDE0259-F321-4AAE-BB08-0BC2E5A737F7}" name="triads_gaze_counts_stats_floorlevel__21216" displayName="triads_gaze_counts_stats_floorlevel__21216" ref="F2:O5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="3">
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{7FDE0259-F321-4AAE-BB08-0BC2E5A737F7}" name="triads_gaze_counts_stats_floorlevel__21216" displayName="triads_gaze_counts_stats_floorlevel__21216" ref="F2:O5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="7">
   <autoFilter ref="F2:O5" xr:uid="{240E3FA1-9A53-416B-84DD-756B154FEAB1}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{F4E1600F-545A-4249-B39A-437021776FD3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{F4E1600F-545A-4249-B39A-437021776FD3}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{F7E4BB1A-1081-423B-B73B-991F08FD0697}" uniqueName="2" name="Percentage_0_D1" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{22364F8F-4EDD-4D31-A8D7-15963C0A85C2}" uniqueName="3" name="Percentage_1_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{522654CA-D0D9-40EC-B2EA-7804300F44A8}" uniqueName="4" name="Percentage_2_D1_same" queryTableFieldId="4"/>
@@ -542,11 +655,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{9D6B5AA9-E372-4765-B2BD-764D74D5FB9B}" name="triads_gaze_counts_stats1317" displayName="triads_gaze_counts_stats1317" ref="F11:O14" tableType="queryTable" totalsRowShown="0" headerRowDxfId="1">
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{9D6B5AA9-E372-4765-B2BD-764D74D5FB9B}" name="triads_gaze_counts_stats1317" displayName="triads_gaze_counts_stats1317" ref="F11:O14" tableType="queryTable" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="F11:O14" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{881A3E44-7CB3-4944-8559-CA4EE2EA2E13}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{881A3E44-7CB3-4944-8559-CA4EE2EA2E13}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{3CDAEE36-837E-4B6E-8043-AE0AAF1962E5}" uniqueName="2" name="Percentage_0_D1" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{D27C4B7A-1239-483B-B6C8-136258642351}" uniqueName="3" name="Percentage_1_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{6783D23F-046F-4892-8EF0-835A4EAF1471}" uniqueName="4" name="Percentage_2_D1_same" queryTableFieldId="4"/>
@@ -565,7 +678,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{4DD56BF8-FF38-4FA2-B8B4-490F1D584758}" name="dyads_gaze_counts_stats" displayName="dyads_gaze_counts_stats" ref="A1:D9" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D9" xr:uid="{4DD56BF8-FF38-4FA2-B8B4-490F1D584758}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D2E21794-DFAC-48D7-A038-89C2DEA581B6}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{D2E21794-DFAC-48D7-A038-89C2DEA581B6}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="22"/>
     <tableColumn id="2" xr3:uid="{DBA908F5-E41B-456F-B301-C782EF0E4CE0}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{84543BB1-FC5A-49E9-B237-CB39ED05E15E}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{F83C6929-DFBA-4924-A184-D85F06A1E0A2}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
@@ -578,7 +691,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5AB0FDC6-EA0A-473A-AEC1-526F42A28575}" name="triads_gaze_counts_stats_floorlevel__2" displayName="triads_gaze_counts_stats_floorlevel__2" ref="A1:J9" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:J9" xr:uid="{5AB0FDC6-EA0A-473A-AEC1-526F42A28575}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{5A64CFDD-F9C3-471D-BEB8-053BD5C9D791}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{5A64CFDD-F9C3-471D-BEB8-053BD5C9D791}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="21"/>
     <tableColumn id="2" xr3:uid="{472FCBAD-A1EE-4CDE-8B2B-B4B97E377A27}" uniqueName="2" name="Percentage_0_D1" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{8FD1B5D9-157A-48B9-A757-1875D946A0D5}" uniqueName="3" name="Percentage_1_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{F85B0ADB-04DB-4B48-9D0E-9723E4D25005}" uniqueName="4" name="Percentage_2_D1_same" queryTableFieldId="4"/>
@@ -597,7 +710,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{47CF8148-5325-47B4-8ACC-0F9D8D4CE9F4}" name="triads_gaze_counts_stats" displayName="triads_gaze_counts_stats" ref="A1:J9" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:J9" xr:uid="{47CF8148-5325-47B4-8ACC-0F9D8D4CE9F4}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{1EFE24A2-1603-444A-ABA4-22BBAD7E2F78}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{1EFE24A2-1603-444A-ABA4-22BBAD7E2F78}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="20"/>
     <tableColumn id="2" xr3:uid="{17D5AF2B-2256-419A-9460-03CA9B228823}" uniqueName="2" name="Percentage_0_D1" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{80F788B8-5D50-4C04-A84A-33D0A9A57D4E}" uniqueName="3" name="Percentage_1_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{2425AEC0-E7E6-4792-82E6-621A203241FD}" uniqueName="4" name="Percentage_2_D1_same" queryTableFieldId="4"/>
@@ -613,10 +726,10 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{53B72080-B5EF-4656-81C3-34F5EEA880E8}" name="dyads_gaze_counts_stats_floorlevel__210" displayName="dyads_gaze_counts_stats_floorlevel__210" ref="A2:D10" tableType="queryTable" totalsRowShown="0" headerRowDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{53B72080-B5EF-4656-81C3-34F5EEA880E8}" name="dyads_gaze_counts_stats_floorlevel__210" displayName="dyads_gaze_counts_stats_floorlevel__210" ref="A2:D10" tableType="queryTable" totalsRowShown="0" headerRowDxfId="19">
   <autoFilter ref="A2:D10" xr:uid="{53B72080-B5EF-4656-81C3-34F5EEA880E8}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{953E2D44-8F06-4222-8A0A-ABE3CE59B73F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{953E2D44-8F06-4222-8A0A-ABE3CE59B73F}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="18"/>
     <tableColumn id="2" xr3:uid="{EECE8063-BDB3-4997-86C8-D00F83111AF3}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{A104EF7A-1006-4DB7-A4CF-731008D0FE4C}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{ACAC7110-71BD-4D98-A7EB-05A52770D433}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
@@ -626,10 +739,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}" name="dyads_gaze_counts_stats11" displayName="dyads_gaze_counts_stats11" ref="A26:D34" tableType="queryTable" totalsRowShown="0" headerRowDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}" name="dyads_gaze_counts_stats11" displayName="dyads_gaze_counts_stats11" ref="A26:D34" tableType="queryTable" totalsRowShown="0" headerRowDxfId="17">
   <autoFilter ref="A26:D34" xr:uid="{BAFF6665-9A8B-4861-97F9-08AFB4E618AA}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{697A5396-42F9-401E-A8FF-32794083AD51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{697A5396-42F9-401E-A8FF-32794083AD51}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{1E92647F-C79B-46E0-A9E8-E79474C1F8D7}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{4F41DE5F-1227-4A42-8C3D-39567CF15605}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{6A73DFB1-9A33-4A25-8F4D-3EC6B8A3829E}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
@@ -639,10 +752,10 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{240E3FA1-9A53-416B-84DD-756B154FEAB1}" name="triads_gaze_counts_stats_floorlevel__212" displayName="triads_gaze_counts_stats_floorlevel__212" ref="F2:O10" tableType="queryTable" totalsRowShown="0" headerRowDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{240E3FA1-9A53-416B-84DD-756B154FEAB1}" name="triads_gaze_counts_stats_floorlevel__212" displayName="triads_gaze_counts_stats_floorlevel__212" ref="F2:O10" tableType="queryTable" totalsRowShown="0" headerRowDxfId="15">
   <autoFilter ref="F2:O10" xr:uid="{240E3FA1-9A53-416B-84DD-756B154FEAB1}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{E0659C03-95D2-49C7-A548-34B5B11C3D46}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{E0659C03-95D2-49C7-A548-34B5B11C3D46}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="14"/>
     <tableColumn id="2" xr3:uid="{284FE207-4A5E-491F-91D5-10BF58C0EAA5}" uniqueName="2" name="Percentage_0_D1" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{BAD9E67B-1298-49C7-A0F1-0E1E60133DF8}" uniqueName="3" name="Percentage_1_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{7C0066FF-1242-43B3-A17D-CB345EAB2465}" uniqueName="4" name="Percentage_2_D1_same" queryTableFieldId="4"/>
@@ -658,10 +771,10 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}" name="triads_gaze_counts_stats13" displayName="triads_gaze_counts_stats13" ref="F26:O34" tableType="queryTable" totalsRowShown="0" headerRowDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}" name="triads_gaze_counts_stats13" displayName="triads_gaze_counts_stats13" ref="F26:O34" tableType="queryTable" totalsRowShown="0" headerRowDxfId="13">
   <autoFilter ref="F26:O34" xr:uid="{79D29B45-595C-4585-B642-1EDAE38A7A67}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{A7232138-1AD4-4B88-874C-14C2C1081AAF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{A7232138-1AD4-4B88-874C-14C2C1081AAF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{0DA2B8B9-D9BD-4701-9A31-6287F8DD3C87}" uniqueName="2" name="Percentage_0_D1" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{48F60B1C-5E6F-402C-942C-A626BCE00031}" uniqueName="3" name="Percentage_1_D1" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{4F2DC2BD-237D-4EE8-80E5-C2116F0FDC32}" uniqueName="4" name="Percentage_2_D1_same" queryTableFieldId="4"/>
@@ -677,15 +790,15 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{2D8EF511-1FB5-478B-A6CA-0226811E1394}" name="dyads_gaze_counts_stats_floorlevel__21014" displayName="dyads_gaze_counts_stats_floorlevel__21014" ref="A2:D5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="7">
-  <autoFilter ref="A2:D5" xr:uid="{53B72080-B5EF-4656-81C3-34F5EEA880E8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9890FDDC-BCA9-49BB-BF48-F6E962B9AF22}" name="Table1" displayName="Table1" ref="A12:D20" totalsRowShown="0">
+  <autoFilter ref="A12:D20" xr:uid="{9890FDDC-BCA9-49BB-BF48-F6E962B9AF22}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{BE4F5318-5C8B-45DA-8032-5DADA7840162}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{2652FEA9-5E73-4A5C-B6C8-113038188438}" uniqueName="2" name="Percentage_MG_P" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{7958EAAE-9C2F-413B-9BD5-DB1D396EB51B}" uniqueName="3" name="Percentage_0_D1" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{3B2C7F5F-2941-4CD0-8CA3-F1750712FF7F}" uniqueName="4" name="Percentage_1d_DG" queryTableFieldId="4"/>
+    <tableColumn id="1" xr3:uid="{79D49276-07D2-41F0-86E3-C3197F4809DF}" name="Dyads Task Engagement" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{D4ABBE77-E69E-4C1C-8C1F-072288CAC6A3}" name="MG"/>
+    <tableColumn id="3" xr3:uid="{74C4DCBF-DF58-4A53-A837-09A5A917BC73}" name="0_D1"/>
+    <tableColumn id="4" xr3:uid="{13AA9E24-2506-42CB-BAA3-9F28695BA717}" name="1_D1"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1918,14 +2031,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7E8B623-2092-483D-AE1D-203C7F8C0744}">
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.08984375" customWidth="1"/>
+    <col min="6" max="6" width="22.26953125" customWidth="1"/>
     <col min="7" max="8" width="17.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.90625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25.7265625" bestFit="1" customWidth="1"/>
@@ -1936,24 +2049,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="F1" s="3" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="F1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
     </row>
     <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -2352,11 +2465,41 @@
       </c>
     </row>
     <row r="12" spans="1:15" ht="29" x14ac:dyDescent="0.35">
-      <c r="A12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>22</v>
+      <c r="A12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" t="s">
+        <v>28</v>
+      </c>
+      <c r="K12" t="s">
+        <v>29</v>
+      </c>
+      <c r="L12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M12" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.35">
@@ -2370,7 +2513,7 @@
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F13" t="s">
         <v>0</v>
@@ -2512,7 +2655,7 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A17" s="6">
+      <c r="A17" s="4">
         <v>0.25</v>
       </c>
       <c r="B17">
@@ -2524,7 +2667,7 @@
       <c r="D17">
         <v>0.49196000000000001</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="4">
         <v>0.25</v>
       </c>
       <c r="G17">
@@ -2550,7 +2693,7 @@
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A18" s="6">
+      <c r="A18" s="4">
         <v>0.5</v>
       </c>
       <c r="B18">
@@ -2562,7 +2705,7 @@
       <c r="D18">
         <v>0.50947900000000002</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="4">
         <v>0.5</v>
       </c>
       <c r="G18">
@@ -2588,7 +2731,7 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A19" s="6">
+      <c r="A19" s="4">
         <v>0.75</v>
       </c>
       <c r="B19">
@@ -2600,7 +2743,7 @@
       <c r="D19">
         <v>0.52699799999999997</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="4">
         <v>0.75</v>
       </c>
       <c r="G19">
@@ -2664,24 +2807,24 @@
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="F25" s="3" t="s">
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="F25" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
-      <c r="M25" s="4"/>
-      <c r="N25" s="4"/>
-      <c r="O25" s="4"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
     </row>
     <row r="26" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
@@ -3077,6 +3220,387 @@
       </c>
       <c r="O34">
         <v>0.71075690561628979</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A43" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B43" t="s">
+        <v>24</v>
+      </c>
+      <c r="C43" t="s">
+        <v>25</v>
+      </c>
+      <c r="D43" t="s">
+        <v>26</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G43" t="s">
+        <v>25</v>
+      </c>
+      <c r="H43" t="s">
+        <v>26</v>
+      </c>
+      <c r="I43" t="s">
+        <v>27</v>
+      </c>
+      <c r="J43" t="s">
+        <v>28</v>
+      </c>
+      <c r="K43" t="s">
+        <v>29</v>
+      </c>
+      <c r="L43" t="s">
+        <v>30</v>
+      </c>
+      <c r="M43" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>0</v>
+      </c>
+      <c r="B44">
+        <v>7</v>
+      </c>
+      <c r="C44">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
+        <v>22</v>
+      </c>
+      <c r="F44" t="s">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>12</v>
+      </c>
+      <c r="H44">
+        <v>12</v>
+      </c>
+      <c r="I44">
+        <v>12</v>
+      </c>
+      <c r="J44">
+        <v>11</v>
+      </c>
+      <c r="K44">
+        <v>9</v>
+      </c>
+      <c r="L44">
+        <v>10</v>
+      </c>
+      <c r="M44">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B45" s="7">
+        <v>0.521034</v>
+      </c>
+      <c r="C45" s="7">
+        <v>0.46625</v>
+      </c>
+      <c r="D45" s="7">
+        <v>0.50947900000000002</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G45" s="7">
+        <v>0.41084100000000001</v>
+      </c>
+      <c r="H45" s="7">
+        <v>0.39891599999999999</v>
+      </c>
+      <c r="I45" s="7">
+        <v>0.38483899999999999</v>
+      </c>
+      <c r="J45" s="7">
+        <v>0.418989</v>
+      </c>
+      <c r="K45" s="7">
+        <v>0.42510700000000001</v>
+      </c>
+      <c r="L45" s="7">
+        <v>0.45119999999999999</v>
+      </c>
+      <c r="M45" s="7">
+        <v>0.42182900000000001</v>
+      </c>
+      <c r="N45" s="2"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="8">
+        <v>0.15657799999999999</v>
+      </c>
+      <c r="C46" s="8">
+        <v>0.158251</v>
+      </c>
+      <c r="D46" s="8">
+        <v>4.9550999999999998E-2</v>
+      </c>
+      <c r="F46" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="8">
+        <v>0.151505</v>
+      </c>
+      <c r="H46" s="8">
+        <v>0.132773</v>
+      </c>
+      <c r="I46" s="8">
+        <v>0.15337999999999999</v>
+      </c>
+      <c r="J46" s="8">
+        <v>0.155973</v>
+      </c>
+      <c r="K46" s="8">
+        <v>0.21804999999999999</v>
+      </c>
+      <c r="L46" s="8">
+        <v>0.168716</v>
+      </c>
+      <c r="M46" s="8">
+        <v>0.12395399999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" s="8">
+        <v>0.308894</v>
+      </c>
+      <c r="C47" s="8">
+        <v>0.21893099999999999</v>
+      </c>
+      <c r="D47" s="8">
+        <v>0.474441</v>
+      </c>
+      <c r="F47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G47" s="8">
+        <v>8.0060000000000006E-2</v>
+      </c>
+      <c r="H47" s="8">
+        <v>0.113082</v>
+      </c>
+      <c r="I47" s="8">
+        <v>3.5699000000000002E-2</v>
+      </c>
+      <c r="J47" s="8">
+        <v>0.129576</v>
+      </c>
+      <c r="K47" s="8">
+        <v>1.5138E-2</v>
+      </c>
+      <c r="L47" s="8">
+        <v>0.15440100000000001</v>
+      </c>
+      <c r="M47" s="8">
+        <v>0.15896199999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A48" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="B48" s="8">
+        <v>0.43718699999999999</v>
+      </c>
+      <c r="C48" s="8">
+        <v>0.35931800000000003</v>
+      </c>
+      <c r="D48" s="8">
+        <v>0.49196000000000001</v>
+      </c>
+      <c r="F48" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="G48" s="8">
+        <v>0.311083</v>
+      </c>
+      <c r="H48" s="8">
+        <v>0.32530500000000001</v>
+      </c>
+      <c r="I48" s="8">
+        <v>0.35852899999999999</v>
+      </c>
+      <c r="J48" s="8">
+        <v>0.34237499999999998</v>
+      </c>
+      <c r="K48" s="8">
+        <v>0.35978100000000002</v>
+      </c>
+      <c r="L48" s="8">
+        <v>0.326345</v>
+      </c>
+      <c r="M48" s="8">
+        <v>0.36621399999999998</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A49" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="B49" s="8">
+        <v>0.51513399999999998</v>
+      </c>
+      <c r="C49" s="8">
+        <v>0.52607899999999996</v>
+      </c>
+      <c r="D49" s="8">
+        <v>0.50947900000000002</v>
+      </c>
+      <c r="F49" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="G49" s="8">
+        <v>0.44086500000000001</v>
+      </c>
+      <c r="H49" s="8">
+        <v>0.41766300000000001</v>
+      </c>
+      <c r="I49" s="8">
+        <v>0.42343199999999998</v>
+      </c>
+      <c r="J49" s="8">
+        <v>0.44447399999999998</v>
+      </c>
+      <c r="K49" s="8">
+        <v>0.43415100000000001</v>
+      </c>
+      <c r="L49" s="8">
+        <v>0.474138</v>
+      </c>
+      <c r="M49" s="8">
+        <v>0.42474400000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A50" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="B50" s="8">
+        <v>0.57845899999999995</v>
+      </c>
+      <c r="C50" s="8">
+        <v>0.58607500000000001</v>
+      </c>
+      <c r="D50" s="8">
+        <v>0.52699799999999997</v>
+      </c>
+      <c r="F50" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="G50" s="8">
+        <v>0.49920100000000001</v>
+      </c>
+      <c r="H50" s="8">
+        <v>0.46976899999999999</v>
+      </c>
+      <c r="I50" s="8">
+        <v>0.46191700000000002</v>
+      </c>
+      <c r="J50" s="8">
+        <v>0.516652</v>
+      </c>
+      <c r="K50" s="8">
+        <v>0.55061400000000005</v>
+      </c>
+      <c r="L50" s="8">
+        <v>0.57380200000000003</v>
+      </c>
+      <c r="M50" s="8">
+        <v>0.49937999999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>17</v>
+      </c>
+      <c r="B51" s="8">
+        <v>0.79192099999999999</v>
+      </c>
+      <c r="C51" s="8">
+        <v>0.62071100000000001</v>
+      </c>
+      <c r="D51" s="8">
+        <v>0.54451700000000003</v>
+      </c>
+      <c r="F51" t="s">
+        <v>17</v>
+      </c>
+      <c r="G51" s="8">
+        <v>0.62566200000000005</v>
+      </c>
+      <c r="H51" s="8">
+        <v>0.58872800000000003</v>
+      </c>
+      <c r="I51" s="8">
+        <v>0.61673500000000003</v>
+      </c>
+      <c r="J51" s="8">
+        <v>0.67054999999999998</v>
+      </c>
+      <c r="K51" s="8">
+        <v>0.72725600000000001</v>
+      </c>
+      <c r="L51" s="8">
+        <v>0.71662700000000001</v>
+      </c>
+      <c r="M51" s="8">
+        <v>0.61868999999999996</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A52" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B52" s="11">
+        <v>0.26231101549635127</v>
+      </c>
+      <c r="C52" s="11">
+        <v>0.41657942882564714</v>
+      </c>
+      <c r="D52" s="11">
+        <v>0.32110955567800142</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G52" s="10">
+        <v>0.50104232422697093</v>
+      </c>
+      <c r="H52" s="10">
+        <v>0.34624040590083749</v>
+      </c>
+      <c r="I52" s="10">
+        <v>4.92982431295916E-2</v>
+      </c>
+      <c r="J52" s="10">
+        <v>4.5391747969872054E-2</v>
+      </c>
+      <c r="K52" s="10">
+        <v>3.0321223225744172E-3</v>
+      </c>
+      <c r="L52" s="10">
+        <v>1.0994218039000249E-2</v>
+      </c>
+      <c r="M52" s="10">
+        <v>4.4000938411153039E-2</v>
       </c>
     </row>
   </sheetData>
@@ -3086,13 +3610,18 @@
     <mergeCell ref="F1:O1"/>
     <mergeCell ref="F25:O25"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="4">
+  <tableParts count="8">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3117,24 +3646,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="F1" s="3" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="F1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
     </row>
     <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -3313,24 +3842,24 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="F10" s="3" t="s">
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="F10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">

</xml_diff>